<commit_message>
BRD-13 set rebuilt with the business wording of the archive details message and column (V1092); the pack check no longer allows the former technical message
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-13_Data_Migration/04_BIBS_TestPlan_BRD-13_Data_Migration_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-13_Data_Migration/04_BIBS_TestPlan_BRD-13_Data_Migration_v2.0.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Test Conditions'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Scenarios'!$A$4:$F$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Scenarios'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Cases'!$A$4:$R$226</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Cases'!$A$4:$R$227</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Test Cases'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Coverage'!$A$4:$I$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Coverage'!$4:$4</definedName>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D24" s="12" t="n">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25">
@@ -1083,7 +1083,7 @@
     <row r="36">
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>Source: Data Migration Handbook BRD-13 Data Migration. 44 FRs, 23 BRD IDs, 173 test conditions, 12 scenarios, 222 test cases (117 positive, 105 negative).</t>
+          <t>Source: Data Migration Handbook BRD-13 Data Migration. 44 FRs, 23 BRD IDs, 173 test conditions, 12 scenarios, 223 test cases (117 positive, 106 negative).</t>
         </is>
       </c>
     </row>
@@ -11597,7 +11597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R226"/>
+  <dimension ref="A1:R227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -27921,39 +27921,38 @@
       <c r="L217" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-114: "The legacy details are not valid JSON: &lt;original message&gt;" (MIG_ARCHIVE_DETAIL)
-MSG-DM-115: "The legacy details must be an object of label and value" (MIG_ARCHIVE_DETAIL)
-MSG-DM-116: "Branch &lt;branch code&gt; not found" (MIG_BRANCH_UNKNOWN)
-MSG-DM-117: "Branch &lt;branch&gt; not found" (MIG_BRANCH_UNKNOWN)
-MSG-DM-118: "Branch &lt;code&gt; does not exist in BIBS" (MIG_BRANCH_UNKNOWN)
-MSG-DM-119: "Branch &lt;code&gt; not found" (MIG_BRANCH_UNKNOWN)
-MSG-DM-120: "Client &lt;legacy client&gt; is not migrated" (MIG_C01_NOT_LOADED)
-MSG-DM-121: "Client &lt;legacy client&gt; is not migrated" (MIG_CLIENT_NOT_LOADED)
-MSG-DM-122: "Legacy code &lt;legacy&gt; is not in the approved &lt;set&gt; map" (MIG_CODE_NOT_MAPPED)
-MSG-DM-123: "The legacy code is missing" (MIG_CODE_REQUIRED)
-MSG-DM-124: "The rate has no effective date" (MIG_DATE_REQUIRED)
-MSG-DM-125: "The record has no document date" (MIG_DATE_REQUIRED)
-MSG-DM-126: "The file size is missing" (MIG_DOCUMENT_SIZE)
-MSG-DM-127: "Legacy invoice &lt;legacy no&gt; is not loaded" (MIG_F01_NOT_LOADED)
-MSG-DM-128: "Policy &lt;legacy key&gt; is not among the migrated headers" (MIG_HEADER_NOT_LOADED)
-MSG-DM-129: "Insurer &lt;legacy&gt; is not in the approved INSURER map" (MIG_INSURER_NOT_MAPPED)
-MSG-DM-130: "Invoice &lt;target code&gt; not found" (MIG_INVOICE_MISSING)
-MSG-DM-131: "Code map &lt;set code&gt; names no BIBS list" (MIG_MAP_TARGET)
-MSG-DM-132: "Invoice &lt;legacy key&gt; has no insurer share" (MIG_NO_INSURER)
-MSG-DM-133: "The &lt;column&gt; is missing" (MIG_NUMBER_REQUIRED)
-MSG-DM-134: "Account officer &lt;user&gt; is not in the sales organisation" (MIG_OFFICER_UNKNOWN)
-MSG-DM-135: "Original invoice &lt;legacy parent&gt; is not loaded" (MIG_PARENT_NOT_LOADED)
-MSG-DM-136: "Risk code &lt;legacy code&gt; is not in the approved PRODUCT map" (MIG_PRODUCT_NOT_MAPPED)
-MSG-DM-137: "An advice of &lt;ref&gt; is already loaded" (MIG_RA_DUPLICATE)
-MSG-DM-138: "The sum-insured band &lt;value&gt; is not from-to amounts" (MIG_SI_BAND)
-MSG-DM-139: "Invoice &lt;invoice no&gt; has no snapshot" (MIG_SNAPSHOT_MISSING)
-MSG-DM-140: "Value &lt;code&gt; of list &lt;type&gt; does not exist in BIBS" (MIG_TARGET_MISSING)
-MSG-DM-141: "Unapplied payment &lt;ref&gt; is adjusted with the unapplied payments object" (MIG_TRUEUP_ITEM_KIND)
-MSG-DM-142: "Legacy invoice &lt;ref&gt; is not loaded" (MIG_TRUEUP_ITEM_MISSING)
-MSG-DM-143: "The opening-balance adjustment of batch &lt;batch no&gt; is not approved by the Head of Comptrollership" (MIG_TRUEUP_NOT_APPROVED)
-MSG-DM-144: "The adjustment would take &lt;c&gt; of invoice &lt;ref&gt; below zero; it moved in BIBS since go-live - settle it with Comptrollership" (MIG_TRUEUP_OUT_OF_RANGE)
-MSG-DM-145: "Sales unit &lt;code&gt; does not exist in BIBS" (MIG_UNIT_UNKNOWN)
-MSG-DM-146: "Unapplied item &lt;target code&gt; not found" (MIG_UPP_MISSING)</t>
+MSG-DM-114: "The other legacy fields must be label and value pairs separated by ;, for example Insurer: MAL; Remitted on: 01-Jul-2022" (MIG_ARCHIVE_DETAIL)
+MSG-DM-115: "Branch &lt;branch code&gt; not found" (MIG_BRANCH_UNKNOWN)
+MSG-DM-116: "Branch &lt;branch&gt; not found" (MIG_BRANCH_UNKNOWN)
+MSG-DM-117: "Branch &lt;code&gt; does not exist in BIBS" (MIG_BRANCH_UNKNOWN)
+MSG-DM-118: "Branch &lt;code&gt; not found" (MIG_BRANCH_UNKNOWN)
+MSG-DM-119: "Client &lt;legacy client&gt; is not migrated" (MIG_C01_NOT_LOADED)
+MSG-DM-120: "Client &lt;legacy client&gt; is not migrated" (MIG_CLIENT_NOT_LOADED)
+MSG-DM-121: "Legacy code &lt;legacy&gt; is not in the approved &lt;set&gt; map" (MIG_CODE_NOT_MAPPED)
+MSG-DM-122: "The legacy code is missing" (MIG_CODE_REQUIRED)
+MSG-DM-123: "The rate has no effective date" (MIG_DATE_REQUIRED)
+MSG-DM-124: "The record has no document date" (MIG_DATE_REQUIRED)
+MSG-DM-125: "The file size is missing" (MIG_DOCUMENT_SIZE)
+MSG-DM-126: "Legacy invoice &lt;legacy no&gt; is not loaded" (MIG_F01_NOT_LOADED)
+MSG-DM-127: "Policy &lt;legacy key&gt; is not among the migrated headers" (MIG_HEADER_NOT_LOADED)
+MSG-DM-128: "Insurer &lt;legacy&gt; is not in the approved INSURER map" (MIG_INSURER_NOT_MAPPED)
+MSG-DM-129: "Invoice &lt;target code&gt; not found" (MIG_INVOICE_MISSING)
+MSG-DM-130: "Code map &lt;set code&gt; names no BIBS list" (MIG_MAP_TARGET)
+MSG-DM-131: "Invoice &lt;legacy key&gt; has no insurer share" (MIG_NO_INSURER)
+MSG-DM-132: "The &lt;column&gt; is missing" (MIG_NUMBER_REQUIRED)
+MSG-DM-133: "Account officer &lt;user&gt; is not in the sales organisation" (MIG_OFFICER_UNKNOWN)
+MSG-DM-134: "Original invoice &lt;legacy parent&gt; is not loaded" (MIG_PARENT_NOT_LOADED)
+MSG-DM-135: "Risk code &lt;legacy code&gt; is not in the approved PRODUCT map" (MIG_PRODUCT_NOT_MAPPED)
+MSG-DM-136: "An advice of &lt;ref&gt; is already loaded" (MIG_RA_DUPLICATE)
+MSG-DM-137: "The sum-insured band &lt;value&gt; is not from-to amounts" (MIG_SI_BAND)
+MSG-DM-138: "Invoice &lt;invoice no&gt; has no snapshot" (MIG_SNAPSHOT_MISSING)
+MSG-DM-139: "Value &lt;code&gt; of list &lt;type&gt; does not exist in BIBS" (MIG_TARGET_MISSING)
+MSG-DM-140: "Unapplied payment &lt;ref&gt; is adjusted with the unapplied payments object" (MIG_TRUEUP_ITEM_KIND)
+MSG-DM-141: "Legacy invoice &lt;ref&gt; is not loaded" (MIG_TRUEUP_ITEM_MISSING)
+MSG-DM-142: "The opening-balance adjustment of batch &lt;batch no&gt; is not approved by the Head of Comptrollership" (MIG_TRUEUP_NOT_APPROVED)
+MSG-DM-143: "The adjustment would take &lt;c&gt; of invoice &lt;ref&gt; below zero; it moved in BIBS since go-live - settle it with Comptrollership" (MIG_TRUEUP_OUT_OF_RANGE)
+MSG-DM-144: "Sales unit &lt;code&gt; does not exist in BIBS" (MIG_UNIT_UNKNOWN)
+MSG-DM-145: "Unapplied item &lt;target code&gt; not found" (MIG_UPP_MISSING)</t>
         </is>
       </c>
       <c r="M217" s="12" t="inlineStr">
@@ -28028,7 +28027,7 @@
       <c r="L218" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-149: "This pair is already decided" (MIG_PAIR_DECIDED)</t>
+MSG-DM-148: "This pair is already decided" (MIG_PAIR_DECIDED)</t>
         </is>
       </c>
       <c r="M218" s="12" t="inlineStr">
@@ -28103,11 +28102,11 @@
       <c r="L219" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-152: "A record cannot be authorized by the user who maintained it" (MAKER_CHECKER_VIOLATION)
-MSG-DM-153: "Batch &lt;batch no&gt; is &lt;status&gt;; it has no load to reconcile" (MIG_BATCH_STATUS)
-MSG-DM-154: "This line has no difference to explain" (MIG_LINE_MATCHED)
-MSG-DM-155: "Explain the break before approving it" (MIG_NOT_EXPLAINED)
-MSG-DM-156: "Enter the explanation of the break" (MIG_REASON_REQUIRED)</t>
+MSG-DM-151: "A record cannot be authorized by the user who maintained it" (MAKER_CHECKER_VIOLATION)
+MSG-DM-152: "Batch &lt;batch no&gt; is &lt;status&gt;; it has no load to reconcile" (MIG_BATCH_STATUS)
+MSG-DM-153: "This line has no difference to explain" (MIG_LINE_MATCHED)
+MSG-DM-154: "Explain the break before approving it" (MIG_NOT_EXPLAINED)
+MSG-DM-155: "Enter the explanation of the break" (MIG_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M219" s="12" t="inlineStr">
@@ -28182,16 +28181,16 @@
       <c r="L220" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-159: "The Head of Comptrollership approves or returns the adjustment."
-MSG-DM-160: "The adjustment batch may then be loaded; its journals post into the opening period."
-MSG-DM-161: "The adjustment goes back to the preparer."
-MSG-DM-162: "A record cannot be authorized by the user who maintained it" (MAKER_CHECKER_VIOLATION)
-MSG-DM-163: "Enter the reason for the return" (MIG_REASON_REQUIRED)
-MSG-DM-164: "Batch &lt;batch no&gt; is not a batch of object &lt;object&gt;" (MIG_TRUEUP_BATCH)
-MSG-DM-165: "Opening-balance adjustment &lt;no&gt; already exists" (MIG_TRUEUP_EXISTS)
-MSG-DM-166: "The adjustment number is 1, 2, 3 or F" (MIG_TRUEUP_NO)
-MSG-DM-167: "Opening-balance adjustments apply to the year-end go-live; the cut-over option is B" (MIG_TRUEUP_OPTION)
-MSG-DM-168: "True-up &lt;trueup no&gt; is &lt;status&gt;; it cannot be &lt;action&gt;" (MIG_TRUEUP_STATUS)</t>
+MSG-DM-158: "The Head of Comptrollership approves or returns the adjustment."
+MSG-DM-159: "The adjustment batch may then be loaded; its journals post into the opening period."
+MSG-DM-160: "The adjustment goes back to the preparer."
+MSG-DM-161: "A record cannot be authorized by the user who maintained it" (MAKER_CHECKER_VIOLATION)
+MSG-DM-162: "Enter the reason for the return" (MIG_REASON_REQUIRED)
+MSG-DM-163: "Batch &lt;batch no&gt; is not a batch of object &lt;object&gt;" (MIG_TRUEUP_BATCH)
+MSG-DM-164: "Opening-balance adjustment &lt;no&gt; already exists" (MIG_TRUEUP_EXISTS)
+MSG-DM-165: "The adjustment number is 1, 2, 3 or F" (MIG_TRUEUP_NO)
+MSG-DM-166: "Opening-balance adjustments apply to the year-end go-live; the cut-over option is B" (MIG_TRUEUP_OPTION)
+MSG-DM-167: "True-up &lt;trueup no&gt; is &lt;status&gt;; it cannot be &lt;action&gt;" (MIG_TRUEUP_STATUS)</t>
         </is>
       </c>
       <c r="M220" s="12" t="inlineStr">
@@ -28266,19 +28265,19 @@
       <c r="L221" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-169: "Checklist updated"
-MSG-DM-172: "Recorded"
-MSG-DM-173: "The actual end is recorded and the tasks after it may start."
-MSG-DM-174: "The actual start is recorded; the tasks it depends on must be finished."
-MSG-DM-175: "The cut-over stops and rolls back to the snapshot.&lt;gate&gt;"
-MSG-DM-176: "The task is marked blocked with its reason for the cut-over call."
-MSG-DM-177: "Criterion &lt;criterion no&gt; is measured by the system" (MIG_CRITERION_MEASURED)
-MSG-DM-178: "Give the evidence of the criterion" (MIG_EVIDENCE_REQUIRED)
-MSG-DM-179: "Give the go-live date of the plan" (MIG_GOLIVE_REQUIRED)
-MSG-DM-180: "&lt;unmet&gt; criteria are not met; give the justification of the GO" (MIG_GONOGO_JUSTIFY)
-MSG-DM-181: "Give the reason of the NO-GO" (MIG_REASON_REQUIRED)
-MSG-DM-182: "Give the reason of the block" (MIG_REASON_REQUIRED)
-MSG-DM-183: "Task &lt;dep&gt; must be finished before task &lt;seq&gt;" (MIG_TASK_DEPENDENCY)</t>
+MSG-DM-168: "Checklist updated"
+MSG-DM-171: "Recorded"
+MSG-DM-172: "The actual end is recorded and the tasks after it may start."
+MSG-DM-173: "The actual start is recorded; the tasks it depends on must be finished."
+MSG-DM-174: "The cut-over stops and rolls back to the snapshot.&lt;gate&gt;"
+MSG-DM-175: "The task is marked blocked with its reason for the cut-over call."
+MSG-DM-176: "Criterion &lt;criterion no&gt; is measured by the system" (MIG_CRITERION_MEASURED)
+MSG-DM-177: "Give the evidence of the criterion" (MIG_EVIDENCE_REQUIRED)
+MSG-DM-178: "Give the go-live date of the plan" (MIG_GOLIVE_REQUIRED)
+MSG-DM-179: "&lt;unmet&gt; criteria are not met; give the justification of the GO" (MIG_GONOGO_JUSTIFY)
+MSG-DM-180: "Give the reason of the NO-GO" (MIG_REASON_REQUIRED)
+MSG-DM-181: "Give the reason of the block" (MIG_REASON_REQUIRED)
+MSG-DM-182: "Task &lt;dep&gt; must be finished before task &lt;seq&gt;" (MIG_TASK_DEPENDENCY)</t>
         </is>
       </c>
       <c r="M221" s="12" t="inlineStr">
@@ -28353,8 +28352,8 @@
       <c r="L222" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-185: "The checklist of &lt;system&gt; is already open" (MIG_DECOMMISSION_EXISTS)
-MSG-DM-186: "Give the evidence of the criterion" (MIG_EVIDENCE_REQUIRED)</t>
+MSG-DM-184: "The checklist of &lt;system&gt; is already open" (MIG_DECOMMISSION_EXISTS)
+MSG-DM-185: "Give the evidence of the criterion" (MIG_EVIDENCE_REQUIRED)</t>
         </is>
       </c>
       <c r="M222" s="12" t="inlineStr">
@@ -28429,16 +28428,16 @@
       <c r="L223" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-189: "Give the reason for opening the legacy archive" (MIG_ACCESS_REASON_REQUIRED)
-MSG-DM-190: "Archive record &lt;record type&gt; &lt;legacy key&gt; is already loaded" (MIG_ARCHIVE_EXISTS)
-MSG-DM-191: "Archive record &lt;record type&gt; &lt;legacy key&gt; is not loaded" (MIG_ARCHIVE_RECORD_MISSING)
-MSG-DM-192: "Give a client, policy, invoice, receipt or claim, a record type or a date range" (MIG_CRITERIA_REQUIRED)
-MSG-DM-193: "Give the date as yyyy-MM-dd: &lt;value&gt;" (MIG_DATE_INVALID)
-MSG-DM-194: "The SHA-256 of file &lt;file name&gt; does not match the index" (MIG_DOCUMENT_CHECKSUM)
-MSG-DM-195: "File &lt;file name&gt; is not in the transfer folder" (MIG_DOCUMENT_MISSING)
-MSG-DM-196: "File &lt;file name&gt; has &lt;length&gt; bytes; the index says &lt;size bytes&gt;" (MIG_DOCUMENT_SIZE)
-MSG-DM-197: "&lt;total elements&gt; records match; narrow the search to at most &lt;max&gt; records to export" (MIG_EXPORT_TOO_LARGE)
-MSG-DM-198: "Give the legacy system" (MIG_SOURCE_REQUIRED)</t>
+MSG-DM-188: "Give the reason for opening the legacy archive" (MIG_ACCESS_REASON_REQUIRED)
+MSG-DM-189: "Archive record &lt;record type&gt; &lt;legacy key&gt; is already loaded" (MIG_ARCHIVE_EXISTS)
+MSG-DM-190: "Archive record &lt;record type&gt; &lt;legacy key&gt; is not loaded" (MIG_ARCHIVE_RECORD_MISSING)
+MSG-DM-191: "Give a client, policy, invoice, receipt or claim, a record type or a date range" (MIG_CRITERIA_REQUIRED)
+MSG-DM-192: "Give the date as yyyy-MM-dd: &lt;value&gt;" (MIG_DATE_INVALID)
+MSG-DM-193: "The SHA-256 of file &lt;file name&gt; does not match the index" (MIG_DOCUMENT_CHECKSUM)
+MSG-DM-194: "File &lt;file name&gt; is not in the transfer folder" (MIG_DOCUMENT_MISSING)
+MSG-DM-195: "File &lt;file name&gt; has &lt;length&gt; bytes; the index says &lt;size bytes&gt;" (MIG_DOCUMENT_SIZE)
+MSG-DM-196: "&lt;total elements&gt; records match; narrow the search to at most &lt;max&gt; records to export" (MIG_EXPORT_TOO_LARGE)
+MSG-DM-197: "Give the legacy system" (MIG_SOURCE_REQUIRED)</t>
         </is>
       </c>
       <c r="M223" s="12" t="inlineStr">
@@ -28513,11 +28512,11 @@
       <c r="L224" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-204: "The Cashiering team lead approves first, then top management; the lines post after the second approval."
-MSG-DM-205: "The Cashiering team lead approves; any premium receivable needed is first moved to PR 2307."
-MSG-DM-206: "The Commission team lead approves; each invoice then posts on its own."
-MSG-DM-207: "The batch goes back to its requester as a draft."
-MSG-DM-208: "The batch is closed without posting; its lines may be taken again."</t>
+MSG-DM-203: "The Cashiering team lead approves first, then top management; the lines post after the second approval."
+MSG-DM-204: "The Cashiering team lead approves; any premium receivable needed is first moved to PR 2307."
+MSG-DM-205: "The Commission team lead approves; each invoice then posts on its own."
+MSG-DM-206: "The batch goes back to its requester as a draft."
+MSG-DM-207: "The batch is closed without posting; its lines may be taken again."</t>
         </is>
       </c>
       <c r="M224" s="12" t="inlineStr">
@@ -28580,7 +28579,7 @@
       <c r="L225" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-209: "Checked"</t>
+MSG-DM-208: "Checked"</t>
         </is>
       </c>
       <c r="M225" s="12" t="inlineStr">
@@ -28643,11 +28642,11 @@
       <c r="L226" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-DM-210: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-DM-211: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-DM-212: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-DM-213: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-DM-214: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-DM-209: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-DM-210: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-DM-211: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-DM-212: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-DM-213: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
 MSG-DM-215: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
 MSG-DM-216: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
@@ -28667,12 +28666,75 @@
       <c r="Q226" s="28" t="n"/>
       <c r="R226" s="12" t="n"/>
     </row>
+    <row r="227">
+      <c r="A227" s="12" t="inlineStr">
+        <is>
+          <t>TC-DM-MSG-17</t>
+        </is>
+      </c>
+      <c r="B227" s="12" t="inlineStr"/>
+      <c r="C227" s="12" t="inlineStr"/>
+      <c r="D227" s="12" t="inlineStr"/>
+      <c r="E227" s="12" t="inlineStr">
+        <is>
+          <t>Messages of Several screens</t>
+        </is>
+      </c>
+      <c r="F227" s="12" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="G227" s="12" t="inlineStr">
+        <is>
+          <t>DML – Data Migration Lead</t>
+        </is>
+      </c>
+      <c r="H227" s="12" t="inlineStr">
+        <is>
+          <t>Any Data Migration record</t>
+        </is>
+      </c>
+      <c r="I227" s="12" t="inlineStr"/>
+      <c r="J227" s="12" t="inlineStr">
+        <is>
+          <t>Seed data of the SIT environment.</t>
+        </is>
+      </c>
+      <c r="K227" s="12" t="inlineStr">
+        <is>
+          <t>1. Sign in as -.
+2. Open Any Data Migration record.
+3. For each message listed, create the condition described in the messages catalogue of the Data Migration Handbook (chapter 15) and run the action.</t>
+        </is>
+      </c>
+      <c r="L227" s="12" t="inlineStr">
+        <is>
+          <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
+MSG-DM-214: "There is no layout in force to export" (MIG_NO_LAYOUT)</t>
+        </is>
+      </c>
+      <c r="M227" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N227" s="27" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="O227" s="12" t="n"/>
+      <c r="P227" s="12" t="n"/>
+      <c r="Q227" s="28" t="n"/>
+      <c r="R227" s="12" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:R226"/>
+  <autoFilter ref="A4:R227"/>
   <mergeCells count="1">
     <mergeCell ref="A2:R2"/>
   </mergeCells>
-  <conditionalFormatting sqref="N5:N726">
+  <conditionalFormatting sqref="N5:N727">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Pass"</formula>
     </cfRule>
@@ -28686,19 +28748,19 @@
       <formula>"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:R726">
+  <conditionalFormatting sqref="A5:R727">
     <cfRule type="expression" priority="5" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F5:F726" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="F5:F727" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'_lists'!$B$1:$B$9</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M726" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="M5:M727" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'_lists'!$C$1:$C$3</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N726" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="N5:N727" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'_lists'!$D$1:$D$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>